<commit_message>
Alinear documentación con Guía 2.4: stack definido, Tesseract OCR local y nueva actividad de entorno
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de Documentación/Planificación Inicial/Carta Gantt - TTDH Automation.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de Documentación/Planificación Inicial/Carta Gantt - TTDH Automation.xlsx
@@ -302,7 +302,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table_1" displayName="Table_1" ref="A1:O18" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table_1" displayName="Table_1" ref="A1:O19" headerRowCount="1">
   <tableColumns count="15">
     <tableColumn id="1" name="Actividades / Tareas"/>
     <tableColumn id="2" name="Semana 5"/>
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O18"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="33.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -831,7 +831,7 @@
     <row r="8" ht="38.25" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Recepción por correo y extracción de documentos (OCR/IA)</t>
+          <t>Configuración del entorno de desarrollo y datos simulados</t>
         </is>
       </c>
       <c r="B8" s="7" t="n"/>
@@ -843,11 +843,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="G8" s="7" t="n"/>
       <c r="H8" s="7" t="n"/>
       <c r="I8" s="7" t="n"/>
       <c r="J8" s="7" t="n"/>
@@ -857,17 +853,17 @@
       <c r="N8" s="7" t="n"/>
       <c r="O8" s="7" t="n"/>
     </row>
-    <row r="9" ht="25.5" customHeight="1">
+    <row r="9" ht="38.25" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Implementación del ETL</t>
+          <t>Recepción por correo y extracción de documentos (OCR/IA)</t>
         </is>
       </c>
       <c r="B9" s="7" t="n"/>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="12" t="n"/>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -877,11 +873,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="H9" s="7" t="n"/>
       <c r="I9" s="7" t="n"/>
       <c r="J9" s="7" t="n"/>
       <c r="K9" s="7" t="n"/>
@@ -890,17 +882,17 @@
       <c r="N9" s="7" t="n"/>
       <c r="O9" s="7" t="n"/>
     </row>
-    <row r="10" ht="38.25" customHeight="1">
+    <row r="10" ht="25.5" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Implementación de validaciones y reglas de negocio</t>
+          <t>Implementación del ETL</t>
         </is>
       </c>
       <c r="B10" s="7" t="n"/>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="E10" s="12" t="n"/>
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -910,7 +902,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="H10" s="7" t="n"/>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I10" s="7" t="n"/>
       <c r="J10" s="7" t="n"/>
       <c r="K10" s="7" t="n"/>
@@ -922,25 +918,25 @@
     <row r="11" ht="38.25" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Implementación del componente de IA (detección de anomalías)</t>
+          <t>Implementación de validaciones y reglas de negocio</t>
         </is>
       </c>
       <c r="B11" s="7" t="n"/>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
       <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7" t="n"/>
-      <c r="G11" s="7" t="n"/>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="n"/>
+      <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="n"/>
       <c r="K11" s="7" t="n"/>
       <c r="L11" s="7" t="n"/>
@@ -951,7 +947,7 @@
     <row r="12" ht="38.25" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Comparación histórica y trazabilidad</t>
+          <t>Implementación del componente de IA (detección de anomalías)</t>
         </is>
       </c>
       <c r="B12" s="7" t="n"/>
@@ -965,7 +961,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="I12" s="7" t="n"/>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J12" s="7" t="n"/>
       <c r="K12" s="7" t="n"/>
       <c r="L12" s="7" t="n"/>
@@ -976,7 +976,7 @@
     <row r="13" ht="38.25" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Desarrollo de dashboard y monitoreo</t>
+          <t>Comparación histórica y trazabilidad</t>
         </is>
       </c>
       <c r="B13" s="7" t="n"/>
@@ -985,12 +985,12 @@
       <c r="E13" s="7" t="n"/>
       <c r="F13" s="7" t="n"/>
       <c r="G13" s="7" t="n"/>
-      <c r="H13" s="7" t="n"/>
-      <c r="I13" s="7" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="n"/>
       <c r="J13" s="7" t="n"/>
       <c r="K13" s="7" t="n"/>
       <c r="L13" s="7" t="n"/>
@@ -998,10 +998,10 @@
       <c r="N13" s="7" t="n"/>
       <c r="O13" s="7" t="n"/>
     </row>
-    <row r="14" ht="25.5" customHeight="1">
+    <row r="14" ht="38.25" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Implementación de reportes</t>
+          <t>Desarrollo de dashboard y monitoreo</t>
         </is>
       </c>
       <c r="B14" s="7" t="n"/>
@@ -1026,7 +1026,7 @@
     <row r="15" ht="25.5" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Integración de componentes</t>
+          <t>Implementación de reportes</t>
         </is>
       </c>
       <c r="B15" s="7" t="n"/>
@@ -1036,12 +1036,12 @@
       <c r="F15" s="7" t="n"/>
       <c r="G15" s="7" t="n"/>
       <c r="H15" s="7" t="n"/>
-      <c r="I15" s="7" t="n"/>
-      <c r="J15" s="7" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="n"/>
       <c r="K15" s="7" t="n"/>
       <c r="L15" s="7" t="n"/>
       <c r="M15" s="7" t="n"/>
@@ -1051,7 +1051,7 @@
     <row r="16" ht="25.5" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Pruebas funcionales y de integración</t>
+          <t>Integración de componentes</t>
         </is>
       </c>
       <c r="B16" s="7" t="n"/>
@@ -1062,12 +1062,12 @@
       <c r="G16" s="7" t="n"/>
       <c r="H16" s="7" t="n"/>
       <c r="I16" s="7" t="n"/>
-      <c r="J16" s="7" t="n"/>
-      <c r="K16" s="7" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J16" s="7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K16" s="7" t="n"/>
       <c r="L16" s="7" t="n"/>
       <c r="M16" s="7" t="n"/>
       <c r="N16" s="7" t="n"/>
@@ -1076,7 +1076,7 @@
     <row r="17" ht="25.5" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Correcciones y documentación final</t>
+          <t>Pruebas funcionales y de integración</t>
         </is>
       </c>
       <c r="B17" s="7" t="n"/>
@@ -1088,12 +1088,12 @@
       <c r="H17" s="7" t="n"/>
       <c r="I17" s="7" t="n"/>
       <c r="J17" s="7" t="n"/>
-      <c r="K17" s="7" t="n"/>
-      <c r="L17" s="7" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="K17" s="7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L17" s="7" t="n"/>
       <c r="M17" s="7" t="n"/>
       <c r="N17" s="7" t="n"/>
       <c r="O17" s="7" t="n"/>
@@ -1101,7 +1101,7 @@
     <row r="18" ht="25.5" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Presentación y cierre del proyecto</t>
+          <t>Correcciones y documentación final</t>
         </is>
       </c>
       <c r="B18" s="7" t="n"/>
@@ -1114,18 +1114,43 @@
       <c r="I18" s="7" t="n"/>
       <c r="J18" s="7" t="n"/>
       <c r="K18" s="7" t="n"/>
-      <c r="L18" s="7" t="n"/>
-      <c r="M18" s="7" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="N18" s="7" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O18" s="7" t="inlineStr">
+      <c r="L18" s="7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M18" s="7" t="n"/>
+      <c r="N18" s="7" t="n"/>
+      <c r="O18" s="7" t="n"/>
+    </row>
+    <row r="19" ht="25.5" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Presentación y cierre del proyecto</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="7" t="n"/>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="7" t="n"/>
+      <c r="H19" s="7" t="n"/>
+      <c r="I19" s="7" t="n"/>
+      <c r="J19" s="7" t="n"/>
+      <c r="K19" s="7" t="n"/>
+      <c r="L19" s="7" t="n"/>
+      <c r="M19" s="7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="N19" s="7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O19" s="7" t="inlineStr">
         <is>
           <t>X</t>
         </is>

</xml_diff>